<commit_message>
adding additional imports from CCO
</commit_message>
<xml_diff>
--- a/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
+++ b/ClimOO material/materials for implementations /ClimOO Vocabulary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/f.u./Desktop/ClimOO-Ontology/ClimOO material/materials for implementations /"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644F0F0F-C9D3-7445-AEBA-43BD9FEE45D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B034F02-DB40-A545-B432-80EF90361BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="29520" yWindow="4280" windowWidth="28800" windowHeight="16380" xr2:uid="{CB153552-6711-0040-AB62-F0CB02156726}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2577" uniqueCount="856">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2613" uniqueCount="868">
   <si>
     <t>Terms</t>
   </si>
@@ -2607,6 +2607,42 @@
   </si>
   <si>
     <t>yes</t>
+  </si>
+  <si>
+    <t>optical property</t>
+  </si>
+  <si>
+    <t>electromagnetic radiation property</t>
+  </si>
+  <si>
+    <t>color</t>
+  </si>
+  <si>
+    <t>black</t>
+  </si>
+  <si>
+    <t>blue</t>
+  </si>
+  <si>
+    <t>brown</t>
+  </si>
+  <si>
+    <t>green</t>
+  </si>
+  <si>
+    <t>grey</t>
+  </si>
+  <si>
+    <t>orange</t>
+  </si>
+  <si>
+    <t>white</t>
+  </si>
+  <si>
+    <t>red</t>
+  </si>
+  <si>
+    <t>yellow</t>
   </si>
 </sst>
 </file>
@@ -2686,17 +2722,7 @@
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="4">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="3">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -3057,7 +3083,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A05EE52F-6B9B-9646-8D2F-C9D94D87C781}">
-  <dimension ref="A1:D861"/>
+  <dimension ref="A1:D873"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="82.5" style="1" bestFit="1" customWidth="1"/>
@@ -12514,18 +12540,150 @@
         <v>855</v>
       </c>
     </row>
+    <row r="862" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A862" s="1" t="s">
+        <v>857</v>
+      </c>
+      <c r="B862" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C862" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="863" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A863" s="1" t="s">
+        <v>856</v>
+      </c>
+      <c r="B863" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C863" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="864" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A864" s="1" t="s">
+        <v>858</v>
+      </c>
+      <c r="B864" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C864" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="865" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A865" s="1" t="s">
+        <v>859</v>
+      </c>
+      <c r="B865" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C865" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="866" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A866" s="1" t="s">
+        <v>860</v>
+      </c>
+      <c r="B866" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C866" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="867" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A867" s="1" t="s">
+        <v>861</v>
+      </c>
+      <c r="B867" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C867" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="868" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A868" s="1" t="s">
+        <v>862</v>
+      </c>
+      <c r="B868" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C868" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="869" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A869" s="1" t="s">
+        <v>863</v>
+      </c>
+      <c r="B869" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C869" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="870" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A870" s="1" t="s">
+        <v>864</v>
+      </c>
+      <c r="B870" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C870" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="871" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A871" s="1" t="s">
+        <v>865</v>
+      </c>
+      <c r="B871" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C871" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="872" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A872" s="1" t="s">
+        <v>866</v>
+      </c>
+      <c r="B872" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C872" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
+    <row r="873" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A873" s="1" t="s">
+        <v>867</v>
+      </c>
+      <c r="B873" s="1" t="s">
+        <v>855</v>
+      </c>
+      <c r="C873" s="1" t="s">
+        <v>855</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C226">
     <sortCondition ref="A1:A226"/>
   </sortState>
+  <conditionalFormatting sqref="A1:A1048576">
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A895:A1048576 A1:A739">
-    <cfRule type="duplicateValues" dxfId="2" priority="3"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="3"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="D831:D836">
-    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A1:A1048576">
-    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>